<commit_message>
excel: guardar de verdad (parseo en front + POST /viajes/) y fix de build
- parseExcel lee el .xlsx en el navegador (SheetJS) en vez de asumir endpoints de Excel inexistentes en el backend
- syncExcelRows crea cada viaje seleccionado con createTrip (/viajes/); agencia del usuario logueado
- columna Telefonos en la plantilla y validacion (telefono de pasajero obligatorio)
- fix TS2345 en viajes.ts que rompia el build de Vercel
- docs/api-endpoints.md con los endpoints reales del backend

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/viajes-prueba.xlsx
+++ b/viajes-prueba.xlsx
@@ -397,18 +397,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <cols>
     <col min="1" max="1" width="7.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="34.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="32.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
+    <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="32.83203125" customWidth="1"/>
-    <col min="9" max="9" width="10.83203125" customWidth="1"/>
-    <col min="10" max="10" width="30.83203125" customWidth="1"/>
+    <col min="9" max="9" width="32.83203125" customWidth="1"/>
+    <col min="10" max="10" width="10.83203125" customWidth="1"/>
+    <col min="11" max="11" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,18 +429,21 @@
         <v>Pasajeros</v>
       </c>
       <c r="F1" t="str">
+        <v>Telefonos</v>
+      </c>
+      <c r="G1" t="str">
         <v>Tipo</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Origen</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Destino</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Vuelo</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Observaciones</v>
       </c>
     </row>
@@ -448,7 +452,7 @@
         <v>V1</v>
       </c>
       <c r="B2" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-14</v>
       </c>
       <c r="C2" t="str">
         <v>06:45</v>
@@ -460,18 +464,21 @@
         <v>Homero Simpson</v>
       </c>
       <c r="F2" t="str">
+        <v>+54 11 5010 1010</v>
+      </c>
+      <c r="G2" t="str">
         <v>out</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>Recoleta</v>
       </c>
-      <c r="H2" t="str">
+      <c r="I2" t="str">
         <v>Aeropuerto Ezeiza (EZE)</v>
       </c>
-      <c r="I2" t="str">
+      <c r="J2" t="str">
         <v>AA1010</v>
       </c>
-      <c r="J2" t="str">
+      <c r="K2" t="str">
         <v/>
       </c>
     </row>
@@ -480,7 +487,7 @@
         <v>V2</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-14</v>
       </c>
       <c r="C3" t="str">
         <v>09:15</v>
@@ -492,18 +499,21 @@
         <v>Marge Bouvier | Ned Flanders</v>
       </c>
       <c r="F3" t="str">
+        <v>+54 11 5020 2020 | +54 11 5020 3030</v>
+      </c>
+      <c r="G3" t="str">
         <v>in</v>
       </c>
-      <c r="G3" t="str">
+      <c r="H3" t="str">
         <v>Aeroparque Jorge Newbery (AEP)</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>Hotel Faena</v>
       </c>
-      <c r="I3" t="str">
+      <c r="J3" t="str">
         <v>LA2480</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Cartel: Sr. Flanders</v>
       </c>
     </row>
@@ -512,7 +522,7 @@
         <v>V3</v>
       </c>
       <c r="B4" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-14</v>
       </c>
       <c r="C4" t="str">
         <v>11:30</v>
@@ -524,18 +534,21 @@
         <v>Lisa Simpson | Bart Simpson | Milhouse V.</v>
       </c>
       <c r="F4" t="str">
+        <v>+54 11 5030 1111 | +54 11 5030 2222 | +54 11 5030 3333</v>
+      </c>
+      <c r="G4" t="str">
         <v>otro</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H4" t="str">
         <v>Tigre</v>
       </c>
-      <c r="H4" t="str">
+      <c r="I4" t="str">
         <v>Microcentro</v>
       </c>
-      <c r="I4" t="str">
-        <v/>
-      </c>
       <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>Reservar 3 valijas</v>
       </c>
     </row>
@@ -556,18 +569,21 @@
         <v/>
       </c>
       <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
         <v>otro</v>
       </c>
-      <c r="G5" t="str">
+      <c r="H5" t="str">
         <v>Microcentro</v>
       </c>
-      <c r="H5" t="str">
+      <c r="I5" t="str">
         <v>Puerto Madero</v>
       </c>
-      <c r="I5" t="str">
-        <v/>
-      </c>
       <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v/>
       </c>
     </row>
@@ -576,7 +592,7 @@
         <v>V4</v>
       </c>
       <c r="B6" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-14</v>
       </c>
       <c r="C6" t="str">
         <v>13:00</v>
@@ -588,18 +604,21 @@
         <v>Montgomery Burns</v>
       </c>
       <c r="F6" t="str">
+        <v>+54 11 5040 4040</v>
+      </c>
+      <c r="G6" t="str">
         <v>in</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H6" t="str">
         <v>Aeropuerto Ezeiza (EZE)</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I6" t="str">
         <v>Hotel Alvear</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J6" t="str">
         <v>IB6843</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K6" t="str">
         <v/>
       </c>
     </row>
@@ -620,18 +639,21 @@
         <v/>
       </c>
       <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
         <v>otro</v>
       </c>
-      <c r="G7" t="str">
+      <c r="H7" t="str">
         <v>Hotel Alvear</v>
       </c>
-      <c r="H7" t="str">
+      <c r="I7" t="str">
         <v>San Isidro</v>
       </c>
-      <c r="I7" t="str">
-        <v/>
-      </c>
       <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
         <v/>
       </c>
     </row>
@@ -652,18 +674,21 @@
         <v/>
       </c>
       <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
         <v>out</v>
       </c>
-      <c r="G8" t="str">
+      <c r="H8" t="str">
         <v>San Isidro</v>
       </c>
-      <c r="H8" t="str">
+      <c r="I8" t="str">
         <v>Aeropuerto Ezeiza (EZE)</v>
       </c>
-      <c r="I8" t="str">
+      <c r="J8" t="str">
         <v>IB6844</v>
       </c>
-      <c r="J8" t="str">
+      <c r="K8" t="str">
         <v/>
       </c>
     </row>
@@ -672,7 +697,7 @@
         <v>V5</v>
       </c>
       <c r="B9" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-14</v>
       </c>
       <c r="C9" t="str">
         <v/>
@@ -684,18 +709,21 @@
         <v/>
       </c>
       <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
         <v>otro</v>
       </c>
-      <c r="G9" t="str">
+      <c r="H9" t="str">
         <v>Belgrano</v>
       </c>
-      <c r="H9" t="str">
+      <c r="I9" t="str">
         <v>Palermo</v>
       </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
       <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
         <v>Completar hora y pasajero al cargar</v>
       </c>
     </row>
@@ -704,7 +732,7 @@
         <v>V6</v>
       </c>
       <c r="B10" t="str">
-        <v>2026-06-14</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C10" t="str">
         <v>10:00</v>
@@ -716,18 +744,21 @@
         <v>Apu Nahasapeemapetilon</v>
       </c>
       <c r="F10" t="str">
+        <v>+54 11 5060 6060</v>
+      </c>
+      <c r="G10" t="str">
         <v>disposicion</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Hotel Hilton Puerto Madero</v>
       </c>
       <c r="H10" t="str">
         <v>Hotel Hilton Puerto Madero</v>
       </c>
       <c r="I10" t="str">
-        <v/>
+        <v>Hotel Hilton Puerto Madero</v>
       </c>
       <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
         <v>4 hs a disposición</v>
       </c>
     </row>
@@ -736,7 +767,7 @@
         <v>V7</v>
       </c>
       <c r="B11" t="str">
-        <v>2026-06-14</v>
+        <v>2026-06-15</v>
       </c>
       <c r="C11" t="str">
         <v>16:20</v>
@@ -748,24 +779,27 @@
         <v>Krusty el Payaso</v>
       </c>
       <c r="F11" t="str">
+        <v>+54 11 5070 7070</v>
+      </c>
+      <c r="G11" t="str">
         <v>otro</v>
       </c>
-      <c r="G11" t="str">
+      <c r="H11" t="str">
         <v>Microcentro</v>
       </c>
-      <c r="H11" t="str">
+      <c r="I11" t="str">
         <v>La Boca</v>
       </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
       <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
         <v>Pasajero VIP</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>